<commit_message>
CSCC-1:2019: split subcontrols into separate assessable requirements
Per maintainer review (#4378): each subcontrol is now its own assessable
requirement (depth 4) and a control with subcontrols is a non-assessable header.
Also add the official source PDF link to the library description.

Structure: 4 domains, 21 subdomains, 32 controls (20 headers + 12 assessable),
73 subcontrols -> 85 assessable requirements.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/excel/cscc/cscc-1-2019.xlsx
+++ b/tools/excel/cscc/cscc-1-2019.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NCA Critical Systems Cybersecurity Controls (CSCC-1:2019), the National Cybersecurity Authority's controls for protecting the Kingdom of Saudi Arabia's critical systems. An elevated set extending the Essential Cybersecurity Controls (ECC) for systems whose failure or compromise would have major national impact. 4 main domains / 21 subdomains / 32 controls. Each subdomain carries its official objective; subcontrols are folded into their parent control. Reference: https://nca.gov.sa</t>
+          <t>NCA Critical Systems Cybersecurity Controls (CSCC-1:2019), the National Cybersecurity Authority's controls for protecting the Kingdom of Saudi Arabia's critical systems. An elevated set extending the Essential Cybersecurity Controls (ECC) for systems whose failure or compromise would have major national impact. 4 main domains / 21 subdomains / 32 controls. Each subdomain carries its official objective; each subcontrol is a separate assessable requirement under its parent control. Source: https://cdn.nca.gov.sa/api/public/cms/files/f15af01c-dc59-4281-95e2-03a770655937_Critical-Systems-Cybersecurity-Controls.pdf</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -790,11 +790,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="n">
         <v>3</v>
       </c>
@@ -806,28 +802,28 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>In addition to the controls in ECC subdomain 1-5, cybersecurity risk management methodology must include at least the following: (1) Conducting a cybersecurity risk assessment on critical systems at least once annually. (2) Creating a cybersecurity risk register for critical systems, and reviewing it at least once every month.</t>
+          <t>In addition to the controls in ECC subdomain 1-5, cybersecurity risk management methodology must include at least the following:</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Cybersecurity in Information Technology Project Management</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>To ensure that cybersecurity requirements are included in project management methodology and procedures in order to protect the confidentiality, integrity and availability of information technology assets as per organization policies, and procedures, and related laws and regulations.</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1-2-1-1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Conducting a cybersecurity risk assessment on critical systems at least once annually.</t>
         </is>
       </c>
     </row>
@@ -838,59 +834,55 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1-3-1</t>
+          <t>1-2-1-2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 1-6-2, cybersecurity requirements of project management and asset (information technology) change management of the organization’s critical systems must include at least the following: (1) Conducting a stress test to ensure the capacity of the various components. (2) Ensuring the implementation of business continuity requirements.</t>
+          <t>Creating a cybersecurity risk register for critical systems, and reviewing it at least once every month.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Cybersecurity in Information Technology Project Management</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>To ensure that cybersecurity requirements are included in project management methodology and procedures in order to protect the confidentiality, integrity and availability of information technology assets as per organization policies, and procedures, and related laws and regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="n">
         <v>3</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1-3-2</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>In addition to the subcontrols in ECC control 1-6-3, cybersecurity requirements related to software and application development projects of the organization’s critical systems must include at least the following: (1) Conducting a security source code review before the critical system release. (2) Securing the access, storage, documentation and releases of source code. (3) Securing the authenticated Application Programming Interface (API). (4) Secure and trusted migration of applications from testing environments to production environments, along with deletion of any data, IDs or passwords related to the testing environment before the migration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Periodical Cybersecurity Review and Audit</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>To ensure that cybersecurity controls are implemented and in compliance with organizational policies and procedures, as well as related national and international laws, regulations and agreements.</t>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1-3-1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 1-6-2, cybersecurity requirements of project management and asset (information technology) change management of the organization’s critical systems must include at least the following:</t>
         </is>
       </c>
     </row>
@@ -901,17 +893,17 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1-4-1</t>
+          <t>1-3-1-1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>With reference to ECC control 1-8-1, the organization’s cybersecurity function must review the implementation of CSCC at least once annually.</t>
+          <t>Conducting a stress test to ensure the capacity of the various components.</t>
         </is>
       </c>
     </row>
@@ -922,38 +914,34 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1-4-2</t>
+          <t>1-3-1-2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>With reference to ECC control 1-8-2, the implementation of CSCC must be reviewed by independent parties within the organization, outside the cybersecurity function at least once every three years.</t>
+          <t>Ensuring the implementation of business continuity requirements.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Cybersecurity in Human Resources</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>To ensure that cybersecurity risks and requirements related to personnel (employees and contractors) are managed efficiently prior to employment, during employment and after termination/separation as per organizational policies and procedures, and related laws and regulations.</t>
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1-3-2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 1-6-3, cybersecurity requirements related to software and application development projects of the organization’s critical systems must include at least the following:</t>
         </is>
       </c>
     </row>
@@ -964,55 +952,59 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1-5-1</t>
+          <t>1-3-2-1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 1-9-3, personnel cybersecurity requirements prior to employment must include at least the following: (1) Screening or vetting candidates for working on critical systems. (2) The technical support and development positions for critical systems, must be filled with experienced Saudi professionals.</t>
+          <t>Conducting a security source code review before the critical system release.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Cybersecurity Defense</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1-3-2-2</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Securing the access, storage, documentation and releases of source code.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr"/>
-      <c r="B16" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Asset Management</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>To ensure that the organization has an accurate and detailed inventory of information technology assets in order to support the organization’s cybersecurity and operational requirements to maintain the confidentiality, integrity and availability of information technical assets.</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1-3-2-3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Securing the authenticated Application Programming Interface (API).</t>
         </is>
       </c>
     </row>
@@ -1023,17 +1015,17 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2-1-1</t>
+          <t>1-3-2-4</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>In addition to the controls in ECC subdomain 2-1, cybersecurity requirements for managing information technology assets must include at least the following: (1) Maintaining an annually-updated inventory of critical systems’ assets. (2) Identifying assets owners and involving them in the asset management lifecycle for critical systems.</t>
+          <t>Secure and trusted migration of applications from testing environments to production environments, along with deletion of any data, IDs or passwords related to the testing environment before the migration.</t>
         </is>
       </c>
     </row>
@@ -1044,17 +1036,17 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Identity and Access Management</t>
+          <t>Periodical Cybersecurity Review and Audit</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>To ensure the secure and restricted logical access to information technology assets in order to prevent unauthorized access and allow only authorized access for users which are necessary to accomplish assigned tasks.</t>
+          <t>To ensure that cybersecurity controls are implemented and in compliance with organizational policies and procedures, as well as related national and international laws, regulations and agreements.</t>
         </is>
       </c>
     </row>
@@ -1069,13 +1061,13 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2-2-1</t>
+          <t>1-4-1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-2-3, cybersecurity requirements for identity and access management of critical systems must include at least the following: (1) Prohibiting remote access from outside the Kingdom of Saudi Arabia. (2) Restricting remote access from inside the Kingdom of Saudi Arabia and verifying each access attempt by the organization’s security operations center, and continuously monitoring activities related to remote access. (3) Using multi-factor authentication for all users. (4) Using multi-factor authentication for privileged users, and on systems utilized for managing critical systems stated in control 2-3-1-4. (5) Developing and implementing a high-standard and secure password policy. (6) Utilizing secure methods and algorithms for storing and processing passwords, such as: Hashing functions. (7) Securely managing service accounts for applications and systems, and disabling interactive login from these accounts. (8) Prohibiting direct access and interaction with databases for all users except for database administrators. Users' access and interaction with databases must be through applications only, with consideration given to applying security solutions that limit or prohibit visibility of classified data to database administrators.</t>
+          <t>With reference to ECC control 1-8-1, the organization’s cybersecurity function must review the implementation of CSCC at least once annually.</t>
         </is>
       </c>
     </row>
@@ -1090,13 +1082,13 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2-2-2</t>
+          <t>1-4-2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>With reference to ECC subcontrol 2-2-3-5, user identities and access rights to critical systems must be reviewed at least once every three months.</t>
+          <t>With reference to ECC control 1-8-2, the implementation of CSCC must be reviewed by independent parties within the organization, outside the cybersecurity function at least once every three years.</t>
         </is>
       </c>
     </row>
@@ -1107,59 +1099,55 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Information System and Information Processing Facilities Protection</t>
+          <t>Cybersecurity in Human Resources</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>To ensure the protection of information systems and information processing facilities, (including workstations and infrastructures) against cyber risks.</t>
+          <t>To ensure that cybersecurity risks and requirements related to personnel (employees and contractors) are managed efficiently prior to employment, during employment and after termination/separation as per organizational policies and procedures, and related laws and regulations.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
         <v>3</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2-3-1</t>
+          <t>1-5-1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-3-3, cybersecurity requirements for protecting critical systems and information processing facilities must include at least the following: (1) Whitelisting of application and software operation files that are allowed to execute on servers hosting critical systems. (2) Protecting servers hosting critical systems using end-point protection solutions that are approved by the organization. (3) Applying security patches and updates at least once every month for external and internet-connected critical systems and at least once every three months for internal critical systems, in line with the organization’s approved change managmenet mechanisms. (4) Allocating specific workstations in an isolated network (Management Network), that is isolated from other networks or services (e.g., email service or internet), to be used by highly privileged accounts. (5) Encrypting the network traffic of non-console administrative access for all technical components of critical systems using secure encryption algorithms and protocols. (6) Reviewing critical systems’ configurations and hardening at least once every six months. (7) Reviewing and changing default configurations, and ensuring the removal of hard-coded, backdoor and/or default passwords, where applicable. (8) Protecting systems’ logs and critical files from unauthorized access, tampering, illegitimate modification and/or deletion.</t>
+          <t>In addition to the subcontrols in ECC control 1-9-3, personnel cybersecurity requirements prior to employment must include at least the following:</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>2-4</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Networks Security Management</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the protection of the organization’s network from cyber risks.</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1-5-1-1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Screening or vetting candidates for working on critical systems.</t>
         </is>
       </c>
     </row>
@@ -1170,80 +1158,72 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2-4-1</t>
+          <t>1-5-1-2</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-5-3, cybersecurity requirements of critical systems’ network security management must include at least the following: (1) Logically and/or physically segregating and isolating critical systems' networks. (2) Reviewing firewall rules and access lists, at least once every six months. (3) Prohibiting direct connection between local network devices and critical systems, unless those devices are scanned to ensure they have security controls that meet the acceptable security levels for critical systems. (4) Prohibiting critical systems from connecting to a wireless network. (5) Protecting against Advanced Persistent Threats (APT) at the network layer. (6) Prohibiting connection to the internet for critical systems that provide internal services to the organization and have no strong need to be accessed from outside the organization. (7) Critical systems that provide services to a limited number of organizations (not individuals), shall use networks isolated from the Internet. (8) Protecting against Distributed Denial of Service (DDoS) attacks to limit risks arising from these attacks. (9) Allowing only whitelisting for critical systems’ firewall access lists.</t>
+          <t>The technical support and development positions for critical systems, must be filled with experienced Saudi professionals.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
-      <c r="B25" s="5" t="n">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Cybersecurity Defense</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr"/>
+      <c r="B26" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>2-5</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Mobile Devices Security</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the protection of mobile devices (including laptops, smartphones, tablets) from cyber risks and to ensure the secure handling of the organization’s information (including sensitive information) while utilizing Bring Your Own Device (BYOD) policy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Asset Management</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>To ensure that the organization has an accurate and detailed inventory of information technology assets in order to support the organization’s cybersecurity and operational requirements to maintain the confidentiality, integrity and availability of information technical assets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="n">
         <v>3</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>2-5-1</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>In addition to the subcontrols in ECC control 2-6-3, cybersecurity requirements for mobile devices security and BYOD in the organization must include at least the following: (1) Prohibting access to critical systems from mobile devices except for a temporary period only, after assessing the risks and obtaining the necessary approvals from the cybersecurity function in the organization. (2) Implementing full disk encryption for mobile devices with access to critical systems.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>2-6</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Data and Information Protection</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>To Ensure the confidentiality, integrity and availability of the organization’s data and information as per organizational policies and procedures, and related laws and regulations.</t>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2-1-1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>In addition to the controls in ECC subdomain 2-1, cybersecurity requirements for managing information technology assets must include at least the following:</t>
         </is>
       </c>
     </row>
@@ -1254,80 +1234,76 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2-6-1</t>
+          <t>2-1-1-1</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-7-3, cybersecurity requirements for protecting and handling data and information must include at least the following: (1) Prohibting the use of critical systems’ data in any environment other than production environment, except after applying strict controls for protecting that data, such as: data masking or data scrambling techniques. (2) Classifying all data within critical systems. (3) Protecting classified data of critical systems using data leakage prevention techniques. (4) Identifying retention period for critical systems-associated data, in accordance with relevant legislations. Only required data must be retained in critical systems’ production environments. (5) Prohibting the transfer of any critical systems’ data from production environment to any other environment.</t>
+          <t>Maintaining an annually-updated inventory of critical systems’ assets.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="5" t="n">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2-1-1-2</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Identifying assets owners and involving them in the asset management lifecycle for critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>2-7</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Cryptography</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the proper and efficient use of cryptography to protect information assets as per organizational policies and procedures, and related laws and regulations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Identity and Access Management</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the secure and restricted logical access to information technology assets in order to prevent unauthorized access and allow only authorized access for users which are necessary to accomplish assigned tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="n">
         <v>3</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>2-7-1</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>In addition to the subcontrols in ECC control 2-8-3, cybersecurity requirements for cryptography must include at least the following: (1) Encrypting all critical systems’ data-in-transit. (2) Encrypting all critical systems’ data-at-rest at the level of files, database or certain columns within database. (3) Using secure and up-to-date methods, algorithms, keys and devices in accordance with what NCA issues in this regard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr"/>
-      <c r="B31" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>2-8</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Backup and Recovery Management</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the protection of the organization’s data and information, including information systems and software configurations from cyber risks as per organizational policies and procedures, and related laws and regulations.</t>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2-2-1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-2-3, cybersecurity requirements for identity and access management of critical systems must include at least the following:</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1314,17 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2-8-1</t>
+          <t>2-2-1-1</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-9-3, cybersecurity requirements for backup and recovery management must include at least the following: (1) Scope and coverage of online and offline backups shall cover all critical systems. (2) Performing backup within planned intervals, according to the organization’s risk assessment. NCA recommends performing backup for critical systems on a daily basis. (3) Securing access, storage and transfer of critical systems’ backups and storage media, and protecting it from destruction, unauthorized access or modification.</t>
+          <t>Prohibiting remote access from outside the Kingdom of Saudi Arabia.</t>
         </is>
       </c>
     </row>
@@ -1359,38 +1335,38 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2-8-2</t>
+          <t>2-2-1-2</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>With reference to ECC subcontrol 2-9-3-3, a periodical test must be conducted at least once every three months in order to determine the efficiency of recovering critical systems backups.</t>
+          <t>Restricting remote access from inside the Kingdom of Saudi Arabia and verifying each access attempt by the organization’s security operations center, and continuously monitoring activities related to remote access.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>2-9</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Vulnerabilities Management</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>To ensure timely detection and effective remediation of technical vulnerabilities to prevent or minimize the probability of exploiting these vulnerabilities to launch cyber attacks against the organization.</t>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2-2-1-3</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Using multi-factor authentication for all users.</t>
         </is>
       </c>
     </row>
@@ -1401,17 +1377,17 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2-9-1</t>
+          <t>2-2-1-4</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-10-3, cybersecurity requirements for technical vulnerabilities management of critical systems must include at least the following: (1) Utilizing trusted methods and tools for vulnerabilities assessments. (2) Assessing and remediating vulnerabilities (by installing security updates and patches) on technical components of critical systems at least once every month for external and internet-connected critical systems, and at least once every three months for internal critical systems. (3) Immediately remediating for critical vulnerabilities, in line with change management processes approved by the organization.</t>
+          <t>Using multi-factor authentication for privileged users, and on systems utilized for managing critical systems stated in control 2-3-1-4.</t>
         </is>
       </c>
     </row>
@@ -1422,38 +1398,38 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2-9-2</t>
+          <t>2-2-1-5</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>With reference to ECC subcontrol 2-10-3-1, vulnerabilities assessments must be conducted on critical systems’ technical components at least once every month.</t>
+          <t>Developing and implementing a high-standard and secure password policy.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr"/>
-      <c r="B37" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>2-10</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Penetration Testing</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>To assess and evaluate the efficiency of the organization’s cybersecurity defense capabilities through simulated cyber attacks to discover unknown weaknesses within the technical infrastructure that may lead to a cyber breach.</t>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2-2-1-6</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Utilizing secure methods and algorithms for storing and processing passwords, such as: Hashing functions.</t>
         </is>
       </c>
     </row>
@@ -1464,17 +1440,17 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2-10-1</t>
+          <t>2-2-1-7</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-11-3, cybersecurity requirements for penetration testing on critical systems must include at least the following: (1) Scope of penetration tests must cover all of the critical systems’ technical components and all its internal and external services. (2) Conducting penetration tests by a qualified team.</t>
+          <t>Securely managing service accounts for applications and systems, and disabling interactive login from these accounts.</t>
         </is>
       </c>
     </row>
@@ -1485,101 +1461,97 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2-10-2</t>
+          <t>2-2-1-8</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>With reference to ECC subcontrol 2-11-3-2, penetration tests must be conducted on critical systems at least once every six months.</t>
+          <t>Prohibiting direct access and interaction with databases for all users except for database administrators. Users' access and interaction with databases must be through applications only, with consideration given to applying security solutions that limit or prohibit visibility of classified data to database administrators.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr"/>
-      <c r="B40" s="5" t="n">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2-2-2</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>With reference to ECC subcontrol 2-2-3-5, user identities and access rights to critical systems must be reviewed at least once every three months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>2-11</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Cybersecurity Event Logs and Monitoring Management</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>To ensure timely collection, analysis and monitoring of cybersecurity events for early detection of potential cyber-attacks in order to prevent or minimize the negative impacts on the organization’s operations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>3</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>2-11-1</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>In addition to the subcontrols in ECC control 2-12-3, cybersecurity requirements for event logs and monitoring management for critical systems must include at least the following: (1) Activating cybersecurity event logs on all technical components of critical systems. (2) Activating and monitoring of alerts and event logs related to file integrity management. (3) Monitoring and analyzing user behavior. (4) Monitoring critical systems security events around the clock. (5) Maintaining and protecting critical systems security events logs. The log shall include all details (e.g., time, date, ID and affected system).</t>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Information System and Information Processing Facilities Protection</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the protection of information systems and information processing facilities, (including workstations and infrastructures) against cyber risks.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A42" t="inlineStr"/>
       <c r="B42" t="n">
         <v>3</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2-11-2</t>
+          <t>2-3-1</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>With reference to ECC subcontrol 2-12-3-5, retention period of cybersecurity’s critical systems event logs must be 18 months minimum, in accordance with relevant legislative and regulatory requirements.</t>
+          <t>In addition to the subcontrols in ECC control 2-3-3, cybersecurity requirements for protecting critical systems and information processing facilities must include at least the following:</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr"/>
-      <c r="B43" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Web Application Security</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the protection of Internet-Facing web applications against cyber risk.</t>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>4</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2-3-1-1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Whitelisting of application and software operation files that are allowed to execute on servers hosting critical systems.</t>
         </is>
       </c>
     </row>
@@ -1590,17 +1562,17 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2-12-1</t>
+          <t>2-3-1-2</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 2-15-3, cybersecurity requirements for external web applications for the organization’s critical systems must include at least the following: (1) Secure session management, including session authenticity, session lockout and session timeout. (2) Applying the minimum standards of Open Web Application Security Project (OWASP) Top Ten.</t>
+          <t>Protecting servers hosting critical systems using end-point protection solutions that are approved by the organization.</t>
         </is>
       </c>
     </row>
@@ -1611,38 +1583,38 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2-12-2</t>
+          <t>2-3-1-3</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>With reference to ECC subcontrol 2-15-3-2, multi-tier architecture principle, with mini- mum 3 tiers, must be used.</t>
+          <t>Applying security patches and updates at least once every month for external and internet-connected critical systems and at least once every three months for internal critical systems, in line with the organization’s approved change managmenet mechanisms.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr"/>
-      <c r="B46" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>2-13</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Application Security</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the protection of the critical systems’ internal applications against cyber risks.</t>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>4</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2-3-1-4</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Allocating specific workstations in an isolated network (Management Network), that is isolated from other networks or services (e.g., email service or internet), to be used by highly privileged accounts.</t>
         </is>
       </c>
     </row>
@@ -1653,17 +1625,17 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2-13-1</t>
+          <t>2-3-1-5</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Cybersecurity requirements for critical systems’ internal applications must be defined, documented, and approved.</t>
+          <t>Encrypting the network traffic of non-console administrative access for all technical components of critical systems using secure encryption algorithms and protocols.</t>
         </is>
       </c>
     </row>
@@ -1674,17 +1646,17 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2-13-2</t>
+          <t>2-3-1-6</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>The cybersecurity requirements for critical systems’ internal applications must be implemented.</t>
+          <t>Reviewing critical systems’ configurations and hardening at least once every six months.</t>
         </is>
       </c>
     </row>
@@ -1695,17 +1667,17 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2-13-3</t>
+          <t>2-3-1-7</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>The cybersecurity requirements for critical systems’ internal applications must include at least the following: (1) Adopting multi-tier architecture principle, provided that number of tiers is not less than three. (2) Using secure protocols (e.g., HTTPS). (3) Outlining the acceptable use policy for users. (4) Secure session management, including session authenticity, session lockout and session timeout.</t>
+          <t>Reviewing and changing default configurations, and ensuring the removal of hard-coded, backdoor and/or default passwords, where applicable.</t>
         </is>
       </c>
     </row>
@@ -1716,55 +1688,55 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2-13-4</t>
+          <t>2-3-1-8</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>The cybersecurity requirements for critical systems’ internal applications must be reviewed periodically.</t>
+          <t>Protecting systems’ logs and critical files from unauthorized access, tampering, illegitimate modification and/or deletion.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr"/>
-      <c r="B51" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Cybersecurity Resilience</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr"/>
+      <c r="A51" s="5" t="inlineStr"/>
+      <c r="B51" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Networks Security Management</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the protection of the organization’s network from cyber risks.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr"/>
-      <c r="B52" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Cybersecurity Resilience Aspects of Business Continuity Management (BCM)</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the inclusion of the cybersecurity resiliency requirements within the organization’s business continuity management and to remediate and minimize the impacts on systems, information processing facilities and critical e-services from disasters caused by cybersecurity incidents.</t>
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2-4-1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-5-3, cybersecurity requirements of critical systems’ network security management must include at least the following:</t>
         </is>
       </c>
     </row>
@@ -1775,55 +1747,59 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3-1-1</t>
+          <t>2-4-1-1</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 3-1-3, cybersecurity requirements for business continuity management must include at least the following: (1) Establishing a disaster recovery center for critical systems. (2) Incorporating critical systems within disaster recovery plans. (3) Conducting periodical tests to ensure the efficiency of disaster recovery plans for critical systems, at least once annually. (4) NCA recommends conducting periodical live Disaster Recovery (DR) test for critical systems.</t>
+          <t>Logically and/or physically segregating and isolating critical systems' networks.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr"/>
-      <c r="B54" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Third-Party and Cloud Computing Cybersecurity</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr"/>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>4</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2-4-1-2</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Reviewing firewall rules and access lists, at least once every six months.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr"/>
-      <c r="B55" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>4-1</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Third-Party Cybersecurity</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the protection of assets against cybersecurity risks related to third parties, including outsourcing and managed services as per organizational policies and procedures, and related laws and regulations.</t>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2-4-1-3</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Prohibiting direct connection between local network devices and critical systems, unless those devices are scanned to ensure they have security controls that meet the acceptable security levels for critical systems.</t>
         </is>
       </c>
     </row>
@@ -1834,38 +1810,38 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>4-1-1</t>
+          <t>2-4-1-4</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>In addition to the controls in ECC subdomain 4-1, cybersecurity requirements for contracts and agreements with third-parties must include at least the following: (1) Screening or vetting of outsourcing and managed services companies and personnel who work on critical systems. (2) Outsourcing and managed services of critical systems must rely on Saudi companies and organizations, in accordance with the relevant legislative and regulatory requirements.</t>
+          <t>Prohibiting critical systems from connecting to a wireless network.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="inlineStr"/>
-      <c r="B57" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>4-2</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Cloud Computing and Hosting Cybersecurity</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>To ensure the proper and efficient remediation of cyber risks and the implementation of cybersecurity requirements related to hosting and cloud computing as per organizational policies and procedures, and related laws and regulations. It is also to ensure the protection of the organization’s information technology assets hosted on the cloud or processed/ managed by third parties.</t>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>4</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2-4-1-5</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Protecting against Advanced Persistent Threats (APT) at the network layer.</t>
         </is>
       </c>
     </row>
@@ -1876,17 +1852,1494 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>4-2-1</t>
+          <t>2-4-1-6</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>In addition to the subcontrols in ECC control 4-2-3, cybersecurity requirements related to the use of hosting and cloud computing services must include at least the following: (1) Hosting of critical systems and any part of their technical components must be inside the organization or within cloud computing services provided by government organizations or Saudi companies that are in compliance with NCA’s Cloud Cybersecurity Controls (CCC), taking into account the classification of the hosted data.</t>
+          <t>Prohibiting connection to the internet for critical systems that provide internal services to the organization and have no strong need to be accessed from outside the organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2-4-1-7</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Critical systems that provide services to a limited number of organizations (not individuals), shall use networks isolated from the Internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2-4-1-8</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Protecting against Distributed Denial of Service (DDoS) attacks to limit risks arising from these attacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2-4-1-9</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Allowing only whitelisting for critical systems’ firewall access lists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr"/>
+      <c r="B62" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Mobile Devices Security</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the protection of mobile devices (including laptops, smartphones, tablets) from cyber risks and to ensure the secure handling of the organization’s information (including sensitive information) while utilizing Bring Your Own Device (BYOD) policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2-5-1</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-6-3, cybersecurity requirements for mobile devices security and BYOD in the organization must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2-5-1-1</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Prohibting access to critical systems from mobile devices except for a temporary period only, after assessing the risks and obtaining the necessary approvals from the cybersecurity function in the organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2-5-1-2</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Implementing full disk encryption for mobile devices with access to critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr"/>
+      <c r="B66" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Data and Information Protection</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>To Ensure the confidentiality, integrity and availability of the organization’s data and information as per organizational policies and procedures, and related laws and regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2-6-1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-7-3, cybersecurity requirements for protecting and handling data and information must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2-6-1-1</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Prohibting the use of critical systems’ data in any environment other than production environment, except after applying strict controls for protecting that data, such as: data masking or data scrambling techniques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2-6-1-2</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Classifying all data within critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2-6-1-3</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Protecting classified data of critical systems using data leakage prevention techniques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>4</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2-6-1-4</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Identifying retention period for critical systems-associated data, in accordance with relevant legislations. Only required data must be retained in critical systems’ production environments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>4</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2-6-1-5</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Prohibting the transfer of any critical systems’ data from production environment to any other environment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr"/>
+      <c r="B73" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>2-7</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Cryptography</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the proper and efficient use of cryptography to protect information assets as per organizational policies and procedures, and related laws and regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="n">
+        <v>3</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2-7-1</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-8-3, cybersecurity requirements for cryptography must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>4</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2-7-1-1</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Encrypting all critical systems’ data-in-transit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>4</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2-7-1-2</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Encrypting all critical systems’ data-at-rest at the level of files, database or certain columns within database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>4</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2-7-1-3</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Using secure and up-to-date methods, algorithms, keys and devices in accordance with what NCA issues in this regard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr"/>
+      <c r="B78" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>2-8</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Backup and Recovery Management</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the protection of the organization’s data and information, including information systems and software configurations from cyber risks as per organizational policies and procedures, and related laws and regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2-8-1</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-9-3, cybersecurity requirements for backup and recovery management must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>4</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2-8-1-1</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Scope and coverage of online and offline backups shall cover all critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>4</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2-8-1-2</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Performing backup within planned intervals, according to the organization’s risk assessment. NCA recommends performing backup for critical systems on a daily basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>4</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2-8-1-3</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Securing access, storage and transfer of critical systems’ backups and storage media, and protecting it from destruction, unauthorized access or modification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>3</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2-8-2</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>With reference to ECC subcontrol 2-9-3-3, a periodical test must be conducted at least once every three months in order to determine the efficiency of recovering critical systems backups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr"/>
+      <c r="B84" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>2-9</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Vulnerabilities Management</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>To ensure timely detection and effective remediation of technical vulnerabilities to prevent or minimize the probability of exploiting these vulnerabilities to launch cyber attacks against the organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="n">
+        <v>3</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2-9-1</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-10-3, cybersecurity requirements for technical vulnerabilities management of critical systems must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>4</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2-9-1-1</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Utilizing trusted methods and tools for vulnerabilities assessments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>4</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2-9-1-2</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Assessing and remediating vulnerabilities (by installing security updates and patches) on technical components of critical systems at least once every month for external and internet-connected critical systems, and at least once every three months for internal critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>4</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2-9-1-3</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Immediately remediating for critical vulnerabilities, in line with change management processes approved by the organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>3</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2-9-2</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>With reference to ECC subcontrol 2-10-3-1, vulnerabilities assessments must be conducted on critical systems’ technical components at least once every month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr"/>
+      <c r="B90" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>2-10</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Penetration Testing</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>To assess and evaluate the efficiency of the organization’s cybersecurity defense capabilities through simulated cyber attacks to discover unknown weaknesses within the technical infrastructure that may lead to a cyber breach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="n">
+        <v>3</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2-10-1</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-11-3, cybersecurity requirements for penetration testing on critical systems must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>4</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2-10-1-1</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Scope of penetration tests must cover all of the critical systems’ technical components and all its internal and external services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>4</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2-10-1-2</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Conducting penetration tests by a qualified team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2-10-2</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>With reference to ECC subcontrol 2-11-3-2, penetration tests must be conducted on critical systems at least once every six months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr"/>
+      <c r="B95" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>2-11</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Cybersecurity Event Logs and Monitoring Management</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>To ensure timely collection, analysis and monitoring of cybersecurity events for early detection of potential cyber-attacks in order to prevent or minimize the negative impacts on the organization’s operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="n">
+        <v>3</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2-11-1</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-12-3, cybersecurity requirements for event logs and monitoring management for critical systems must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>4</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2-11-1-1</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Activating cybersecurity event logs on all technical components of critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>4</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2-11-1-2</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Activating and monitoring of alerts and event logs related to file integrity management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>4</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2-11-1-3</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Monitoring and analyzing user behavior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>4</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2-11-1-4</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Monitoring critical systems security events around the clock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>4</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2-11-1-5</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Maintaining and protecting critical systems security events logs. The log shall include all details (e.g., time, date, ID and affected system).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>3</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>2-11-2</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>With reference to ECC subcontrol 2-12-3-5, retention period of cybersecurity’s critical systems event logs must be 18 months minimum, in accordance with relevant legislative and regulatory requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr"/>
+      <c r="B103" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>Web Application Security</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the protection of Internet-Facing web applications against cyber risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr"/>
+      <c r="B104" t="n">
+        <v>3</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2-12-1</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 2-15-3, cybersecurity requirements for external web applications for the organization’s critical systems must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>4</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2-12-1-1</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Secure session management, including session authenticity, session lockout and session timeout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>4</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>2-12-1-2</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Applying the minimum standards of Open Web Application Security Project (OWASP) Top Ten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>3</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2-12-2</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>With reference to ECC subcontrol 2-15-3-2, multi-tier architecture principle, with mini- mum 3 tiers, must be used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr"/>
+      <c r="B108" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>Application Security</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the protection of the critical systems’ internal applications against cyber risks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>3</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>2-13-1</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Cybersecurity requirements for critical systems’ internal applications must be defined, documented, and approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>3</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2-13-2</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>The cybersecurity requirements for critical systems’ internal applications must be implemented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr"/>
+      <c r="B111" t="n">
+        <v>3</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>2-13-3</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>The cybersecurity requirements for critical systems’ internal applications must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>4</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>2-13-3-1</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Adopting multi-tier architecture principle, provided that number of tiers is not less than three.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>4</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>2-13-3-2</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Using secure protocols (e.g., HTTPS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>4</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>2-13-3-3</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Outlining the acceptable use policy for users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>4</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>2-13-3-4</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Secure session management, including session authenticity, session lockout and session timeout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>3</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>2-13-4</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>The cybersecurity requirements for critical systems’ internal applications must be reviewed periodically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr"/>
+      <c r="B117" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Cybersecurity Resilience</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr"/>
+      <c r="B118" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>Cybersecurity Resilience Aspects of Business Continuity Management (BCM)</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the inclusion of the cybersecurity resiliency requirements within the organization’s business continuity management and to remediate and minimize the impacts on systems, information processing facilities and critical e-services from disasters caused by cybersecurity incidents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="n">
+        <v>3</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>3-1-1</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 3-1-3, cybersecurity requirements for business continuity management must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>4</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>3-1-1-1</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Establishing a disaster recovery center for critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>4</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>3-1-1-2</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Incorporating critical systems within disaster recovery plans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>4</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>3-1-1-3</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Conducting periodical tests to ensure the efficiency of disaster recovery plans for critical systems, at least once annually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>4</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>3-1-1-4</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>NCA recommends conducting periodical live Disaster Recovery (DR) test for critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr"/>
+      <c r="B124" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Third-Party and Cloud Computing Cybersecurity</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr"/>
+      <c r="B125" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>Third-Party Cybersecurity</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the protection of assets against cybersecurity risks related to third parties, including outsourcing and managed services as per organizational policies and procedures, and related laws and regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr"/>
+      <c r="B126" t="n">
+        <v>3</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>4-1-1</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>In addition to the controls in ECC subdomain 4-1, cybersecurity requirements for contracts and agreements with third-parties must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>4</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>4-1-1-1</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Screening or vetting of outsourcing and managed services companies and personnel who work on critical systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>4</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>4-1-1-2</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Outsourcing and managed services of critical systems must rely on Saudi companies and organizations, in accordance with the relevant legislative and regulatory requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr"/>
+      <c r="B129" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>Cloud Computing and Hosting Cybersecurity</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>To ensure the proper and efficient remediation of cyber risks and the implementation of cybersecurity requirements related to hosting and cloud computing as per organizational policies and procedures, and related laws and regulations. It is also to ensure the protection of the organization’s information technology assets hosted on the cloud or processed/ managed by third parties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr"/>
+      <c r="B130" t="n">
+        <v>3</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>4-2-1</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>In addition to the subcontrols in ECC control 4-2-3, cybersecurity requirements related to the use of hosting and cloud computing services must include at least the following:</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>4</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>4-2-1-1</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Hosting of critical systems and any part of their technical components must be inside the organization or within cloud computing services provided by government organizations or Saudi companies that are in compliance with NCA’s Cloud Cybersecurity Controls (CCC), taking into account the classification of the hosted data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CSCC-1:2019: fix source typos (managmenet->management, Prohibting->Prohibiting) per #4384 review
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/excel/cscc/cscc-1-2019.xlsx
+++ b/tools/excel/cscc/cscc-1-2019.xlsx
@@ -1593,7 +1593,7 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Applying security patches and updates at least once every month for external and internet-connected critical systems and at least once every three months for internal critical systems, in line with the organization’s approved change managmenet mechanisms.</t>
+          <t>Applying security patches and updates at least once every month for external and internet-connected critical systems and at least once every three months for internal critical systems, in line with the organization’s approved change management mechanisms.</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Prohibting access to critical systems from mobile devices except for a temporary period only, after assessing the risks and obtaining the necessary approvals from the cybersecurity function in the organization.</t>
+          <t>Prohibiting access to critical systems from mobile devices except for a temporary period only, after assessing the risks and obtaining the necessary approvals from the cybersecurity function in the organization.</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Prohibting the use of critical systems’ data in any environment other than production environment, except after applying strict controls for protecting that data, such as: data masking or data scrambling techniques.</t>
+          <t>Prohibiting the use of critical systems’ data in any environment other than production environment, except after applying strict controls for protecting that data, such as: data masking or data scrambling techniques.</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Prohibting the transfer of any critical systems’ data from production environment to any other environment.</t>
+          <t>Prohibiting the transfer of any critical systems’ data from production environment to any other environment.</t>
         </is>
       </c>
     </row>

</xml_diff>